<commit_message>
modif images niv1 et niv3
</commit_message>
<xml_diff>
--- a/quizz_cine.xlsx
+++ b/quizz_cine.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="39">
   <si>
     <t>Niveau 1</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>Retour vers le Futur 3</t>
+  </si>
+  <si>
+    <t>Vampire Diaries</t>
+  </si>
+  <si>
+    <t>Les Razmokets</t>
   </si>
 </sst>
 </file>
@@ -462,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" customWidth="1"/>
@@ -628,13 +634,10 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>14</v>
+      <c r="A14" t="s">
+        <v>38</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -805,25 +808,41 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>37</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>31</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="E29" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="E30" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E31" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>